<commit_message>
【TinyEditor & Assets & Language】给 TinyEditor 新增 C++ Class 菜单项及其功能
</commit_message>
<xml_diff>
--- a/source/Tools/LanguageGenerator/Editor/lang-en-us.xlsx
+++ b/source/Tools/LanguageGenerator/Editor/lang-en-us.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B192"/>
+  <dimension ref="A1:B193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2732,6 +2732,18 @@
         </is>
       </c>
     </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>TXT_CPP_CLASS</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>C++ Class</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>